<commit_message>
Update AIFTax replication package
</commit_message>
<xml_diff>
--- a/Inter_Rater_Analysis/irr_results/AIFTax_IRR_Report.xlsx
+++ b/Inter_Rater_Analysis/irr_results/AIFTax_IRR_Report.xlsx
@@ -550,7 +550,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-29T01:20:20+00:00</t>
+          <t>2026-08-03T14:49:25+00:00</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
         <v>0.8299319727891155</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.7215966206691312</v>
+        <v>0.7215966206691311</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.919693548772859</v>
@@ -1595,7 +1595,7 @@
         <v>0.8299319727891155</v>
       </c>
       <c r="L2" s="9" t="n">
-        <v>0.7215966206691312</v>
+        <v>0.7215966206691311</v>
       </c>
       <c r="M2" s="9" t="n">
         <v>0.919693548772859</v>
@@ -1965,7 +1965,7 @@
         <v>0.87</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>0.8533724340175953</v>
+        <v>0.8533724340175952</v>
       </c>
       <c r="F4" s="9" t="n"/>
       <c r="G4" s="9" t="n"/>
@@ -1998,9 +1998,7 @@
       <c r="D5" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="9" t="n">
-        <v>1</v>
-      </c>
+      <c r="E5" s="9" t="n"/>
       <c r="F5" s="9" t="n"/>
       <c r="G5" s="9" t="n"/>
       <c r="H5" s="6" t="n">
@@ -2312,15 +2310,9 @@
       <c r="D14" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" s="9" t="n">
-        <v>1</v>
-      </c>
+      <c r="E14" s="9" t="n"/>
+      <c r="F14" s="9" t="n"/>
+      <c r="G14" s="9" t="n"/>
       <c r="H14" s="6" t="n">
         <v>0</v>
       </c>

</xml_diff>